<commit_message>
Refactored Connection and settings page now excel fram also starts dataStream
</commit_message>
<xml_diff>
--- a/Gas_Measurment_8_2025.xlsx
+++ b/Gas_Measurment_8_2025.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D157"/>
+  <dimension ref="A1:D304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3283,6 +3283,2652 @@
         </is>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>16:28:35.195</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C158" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>16:28:35.196</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C159" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>16:28:35.197</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C160" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>16:28:35.198</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C161" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>16:28:35.199</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C162" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>16:28:35.200</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C163" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>16:28:35.201</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C164" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>16:28:35.202</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C165" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>16:28:35.203</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C166" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>16:28:35.204</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C167" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>16:28:35.205</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C168" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>16:28:35.206</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C169" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>16:28:35.207</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C170" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>16:28:35.208</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C171" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>16:28:35.209</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C172" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>16:28:35.210</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C173" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>16:28:35.211</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C174" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>16:28:35.212</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C175" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>16:28:35.213</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C176" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>16:28:35.214</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C177" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>16:28:35.215</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C178" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>16:28:35.216</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C179" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>16:28:35.217</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C180" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>16:28:35.218</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C181" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>16:28:35.219</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C182" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>16:28:35.220</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C183" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>16:28:35.221</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C184" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>16:28:35.222</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C185" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>16:28:35.223</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C186" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>16:28:35.224</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C187" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>16:28:35.225</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C188" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>16:28:35.226</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C189" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>16:28:35.227</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C190" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>16:28:35.228</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C191" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>16:28:35.229</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C192" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>16:28:35.230</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C193" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>16:28:35.231</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C194" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>16:28:35.232</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C195" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>16:28:35.233</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C196" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>16:28:35.234</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C197" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>16:28:35.235</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C198" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>16:28:35.236</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C199" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>16:28:35.237</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C200" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>16:28:35.238</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C201" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>16:28:35.239</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C202" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>16:28:35.240</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C203" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>16:28:35.241</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C204" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>16:28:35.242</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C205" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>16:28:35.243</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C206" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>16:28:35.244</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C207" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>16:28:35.245</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C208" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>16:28:35.246</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C209" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>16:28:35.247</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C210" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>16:28:35.248</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C211" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>16:28:35.249</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C212" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>16:28:35.250</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C213" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>16:28:35.251</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C214" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>16:28:35.252</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C215" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>16:28:35.252</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C216" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>16:28:35.253</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C217" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>16:28:35.254</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C218" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>16:28:35.255</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C219" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>16:28:35.256</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C220" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>16:28:35.257</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C221" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>16:28:35.258</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C222" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>16:28:35.259</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C223" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>16:28:35.260</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C224" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>16:28:35.261</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C225" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>16:28:35.262</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C226" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>16:28:35.263</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C227" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>16:28:35.264</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C228" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>16:28:35.265</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C229" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>16:28:35.266</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C230" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>16:28:35.267</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C231" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>16:28:35.268</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C232" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>16:28:35.269</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C233" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>16:28:35.270</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C234" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>16:28:35.271</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C235" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>16:28:35.272</t>
+        </is>
+      </c>
+      <c r="B236" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C236" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>16:28:35.273</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C237" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>16:28:35.274</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C238" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>16:28:35.275</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C239" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>16:28:35.276</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C240" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>16:28:35.277</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C241" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>16:28:35.278</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C242" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>16:28:35.279</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C243" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>16:28:35.280</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C244" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>16:28:35.281</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C245" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>16:28:35.282</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C246" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>16:28:35.283</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C247" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>16:28:35.284</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C248" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>16:28:35.285</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C249" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>16:28:35.286</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C250" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>16:28:35.287</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C251" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>16:28:35.288</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C252" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>16:28:35.289</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C253" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>16:28:35.290</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C254" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>16:28:35.291</t>
+        </is>
+      </c>
+      <c r="B255" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C255" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>16:28:35.292</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C256" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>16:28:35.293</t>
+        </is>
+      </c>
+      <c r="B257" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C257" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>16:28:35.294</t>
+        </is>
+      </c>
+      <c r="B258" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C258" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>16:28:35.295</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C259" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>16:28:35.296</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C260" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>16:28:35.297</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C261" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>16:28:35.298</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C262" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>16:28:35.299</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C263" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>16:28:35.300</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C264" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>16:28:35.301</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C265" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>16:28:35.302</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C266" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>16:28:35.303</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C267" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>16:28:35.304</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C268" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>16:28:35.305</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C269" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>16:28:35.306</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C270" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>16:28:35.307</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C271" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>16:28:35.308</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C272" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>16:28:35.309</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C273" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>16:28:35.310</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C274" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>16:28:35.311</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C275" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>16:28:35.312</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C276" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>16:28:35.313</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C277" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>16:28:35.314</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C278" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>16:28:35.315</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C279" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>16:28:35.316</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C280" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>16:28:35.317</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C281" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>16:28:35.318</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C282" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>16:28:35.319</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C283" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>16:28:35.320</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C284" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>16:28:35.321</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C285" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>16:28:35.322</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C286" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>16:28:35.323</t>
+        </is>
+      </c>
+      <c r="B287" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C287" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>16:28:35.324</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C288" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>16:28:35.325</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C289" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>16:28:35.326</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C290" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>16:28:35.327</t>
+        </is>
+      </c>
+      <c r="B291" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C291" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>16:28:35.328</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C292" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>16:28:35.329</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C293" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>16:28:35.330</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C294" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>16:28:35.331</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C295" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>16:28:35.332</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="C296" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>16:28:35.332</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C297" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>16:28:35.333</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C298" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>16:28:35.334</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C299" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>16:28:35.335</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C300" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>16:28:35.337</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C301" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>16:28:35.338</t>
+        </is>
+      </c>
+      <c r="B302" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C302" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>16:28:35.339</t>
+        </is>
+      </c>
+      <c r="B303" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C303" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>16:28:35.340</t>
+        </is>
+      </c>
+      <c r="B304" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="C304" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>